<commit_message>
Upgrade to format v2: fix UTF-8 name truncation + add test categories
Format changes (backward compatible — game decoder handles v1 and v2):
- Version byte: 1 → 2
- META_SIZE: 88 → 120 bytes
- set_name field: 32 → 64 bytes (supports ~21 Thai characters)
- creator field stays 32 bytes, moved to offset 88

pokker_encoder.py:
- Add _utf8_safe_bytes() to trim at valid UTF-8 boundary (no mid-char cut)
- VERSION = 2, META_SIZE = 120

encoder.html:
- Fix encodeFixed() to trim at UTF-8 boundary instead of hard byte slice
- VERSION = 2, META_SIZE = 120, creator offset 56 → 88

ตัวอย่างการ์ด.xlsx:
- Updated sample cards with mix of existing categories (Question, Drink,
  Command) and new categories (Confession, Roleplay, Trivia, Wildcard)
  for testing that new category buttons appear after import

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ตัวอย่างการ์ด.xlsx
+++ b/ตัวอย่างการ์ด.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="การ์ด" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="การ์ดทดสอบ" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,61 +26,43 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001565C0"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="003F7FB0"/>
+      <color rgb="00C62828"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00D8842F"/>
+      <color rgb="002E7D32"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="007D5FB2"/>
+      <color rgb="00AD1457"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="002F9A93"/>
+      <color rgb="006A1B9A"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00CF5F93"/>
+      <color rgb="0000838F"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="005F9A42"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="004F63B0"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00C9962F"/>
+      <color rgb="00E65100"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -93,8 +75,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="008A6D56"/>
-        <bgColor rgb="008A6D56"/>
+        <fgColor rgb="005D4037"/>
       </patternFill>
     </fill>
   </fills>
@@ -110,43 +91,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -513,17 +485,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ลำดับ</t>
@@ -550,7 +522,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -559,23 +531,23 @@
           <t>Question</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>ทุกคน</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>ถ้าต้องอยู่บนเกาะร้างคนเดียว คุณจะเอาอะไรไปด้วย 3 อย่าง?</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>ถ้าได้เดินทางไปอีกยุคสมัยได้ จะเลือกยุคไหนและทำไม</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>ดื่ม 1 แก้ว</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="28" customHeight="1">
+    <row r="3">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
@@ -584,23 +556,23 @@
           <t>Question</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>คนที่เกิดเดือนล่าสุด</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>สิ่งที่คุณภูมิใจที่สุดในชีวิตคืออะไร?</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>คนที่นั่งขวามือ</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>สิ่งที่อยากทำก่อนอายุ 30 คืออะไร</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>ดื่ม 1 แก้ว</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1">
+    <row r="4">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -609,376 +581,446 @@
           <t>Question</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>คนที่อายุมากที่สุด</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>ถ้าย้อนเวลาได้จะกลับไปแก้ไขอะไร?</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>ดื่ม 2 แก้ว</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="28" customHeight="1">
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>ทุกคน</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>ถ้ามีพลังพิเศษได้หนึ่งอย่าง จะเลือกอะไร</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>คนตอบสั้นสุดดื่ม 2 แก้ว</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Command</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>คนที่นั่งซ้ายมือ</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>โทรหาแม่แล้วบอกรัก</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Drink</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>คนอายุมากที่สุด</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ดื่มให้กับคนที่ชอบที่สุดในวงนี้</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>ดื่ม 2 แก้ว</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="28" customHeight="1">
+    <row r="6">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Command</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>คนที่ตัวสูงที่สุด</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>ร้องเพลงท่อนฮุกของเพลงที่ชอบที่สุด</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>ดื่ม 2 แก้ว</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="28" customHeight="1">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Drink</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ทุกคน</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ทุกคนดื่มพร้อมกัน นับ 3 2 1</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>ดื่ม 1 แก้ว</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Command</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>คนที่ผมยาวที่สุด</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>เต้นให้ดู 15 วินาที</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>ดื่ม 1 แก้ว</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="28" customHeight="1">
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>คนที่นั่งซ้ายมือ</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>โทรหาผู้ปกครองแล้วบอกรัก</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>ดื่ม 3 แก้ว ถ้าไม่ทำ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Deeptalk</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Command</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>ทุกคน</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>สิ่งที่คุณอยากบอกตัวเองในอดีตมากที่สุดคืออะไร?</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>เล่าให้ฟัง</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="28" customHeight="1">
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>ทุกคนโพสต์สเตตัส emoji เดียว ภายใน 1 นาที</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>ใครไม่โพสต์ดื่ม 2 แก้ว</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Deeptalk</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>คนที่อายุน้อยที่สุด</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>ความฝันที่ยังไม่ได้ทำให้เป็นจริงคืออะไร?</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>เล่าให้ฟัง</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="28" customHeight="1">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Confession</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ทุกคน</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>เล่าเรื่องที่เขินที่สุดในชีวิต</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>ดื่ม 2 แก้ว</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Drink</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>ตัวเอง</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>ดื่ม 3 แก้ว ไม่มีเงื่อนไข</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11" ht="28" customHeight="1">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Confession</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>คนอายุมากที่สุด</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>เคยโกหกใครในวงนี้ไหม? ถ้าเคยให้เล่า</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>ดื่ม 1 แก้ว</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Drink</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>คนที่ผมสั้นที่สุด</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>ดื่ม 2 แก้ว</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12" ht="28" customHeight="1">
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Confession</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>คนที่นั่งซ้ายมือ</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>สิ่งที่เคยทำแล้วยังรู้สึกผิดจนถึงตอนนี้</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>เล่าให้ฟัง 1 นาที</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Skinship</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>คนตรงข้าม</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>จับมือกัน 10 วินาที</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>ดื่ม 1 แก้ว</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Roleplay</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>คนอายุน้อยที่สุด</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>สวมบทเป็นนายกฯ แถลงข่าว 30 วินาที</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>ทำก่อนค่อยดื่ม 1 แก้ว</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>Skinship</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>คนที่นั่งขวามือ</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>โอบไหล่กัน 5 วินาที</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>ดื่ม 1 แก้ว</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Roleplay</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>ทุกคน</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>ทุกคนต้องพูดสำเนียงภาคเหนือจนกว่าจะจั่วใบต่อไป</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>ใครพลาดดื่ม 2 แก้ว</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Minigame</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>ทุกคน</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>เล่น Rock Paper Scissors ผู้แพ้รับโทษ</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>ผู้แพ้ดื่ม 2 แก้ว</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Roleplay</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>คนที่นั่งตรงข้าม</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>สวมบทเป็นพิธีกรแล้วสัมภาษณ์คนข้างๆ</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>ดื่ม 1 แก้ว ถ้าหยุดกลางคัน</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Minigame</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Trivia</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>ทุกคน</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>นับ 1-21 ห้ามพูดเลข 7 กับ 14 ผิดรับโทษ</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>ผู้ผิดดื่ม 1 แก้ว</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="28" customHeight="1">
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>เมืองหลวงของออสเตรเลียคือเมืองอะไร? ใครตอบถูกก่อน</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>คนตอบผิดดื่ม 2 แก้ว</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>Secret</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>คนที่เลือก</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>แอบชอบใครในวงนี้ไหม? ตอบตรงๆ</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>ดื่ม 3 แก้วถ้าโกหก</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="28" customHeight="1">
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Trivia</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>คนที่นั่งขวามือ</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>ถามคำถามข้อเท็จจริง 1 ข้อ ถ้าตอบผิดต้องดื่ม</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>ดื่ม 2 แก้ว</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>Secret</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Trivia</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>ทุกคน</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>บอก Never Have I Ever แล้วคนที่เคยทำดื่ม</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18" ht="28" customHeight="1">
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>ใครนับหนึ่งถึงสิบภาษาญี่ปุ่นได้ครบไม่ต้องดื่ม</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>นับผิดดื่ม 1 แก้ว</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>Special</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>ทุกคน</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>ทุกคนดื่มพร้อมกัน 1 แก้ว แล้วเล่าความลับ 1 เรื่อง</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19" ht="28" customHeight="1">
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Wildcard</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>คนที่จั่วใบนี้</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>เลือกกฎใหม่ 1 ข้อใช้ตลอดรอบนี้</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>ไม่เลือกภายใน 10 วินาทีดื่ม 3 แก้ว</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>Special</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>คนที่เลือก</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>ตั้งกฎใหม่ของวงที่ทุกคนต้องทำจนครบรอบ</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr"/>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Wildcard</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>ทุกคน</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>สับใหม่! ทุกคนดื่มพร้อมกัน 1 แก้ว แล้วเริ่มใหม่</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>ดื่ม 1 แก้ว</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Wildcard</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>คนที่นั่งตรงข้าม</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>สลับที่นั่งกับคนใดก็ได้ในวง</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>ถ้าไม่สลับดื่ม 2 แก้ว</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Wildcard</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>คนอายุมากที่สุด</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>กำหนดว่าใครดื่มแทนใครในรอบถัดไป</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>ปฏิเสธดื่มเอง 3 แก้ว</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>